<commit_message>
removed unnecessary field from the  report
</commit_message>
<xml_diff>
--- a/reports/sample/sample-monthly-ip-report.xlsx
+++ b/reports/sample/sample-monthly-ip-report.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t xml:space="preserve">SBU</t>
   </si>
@@ -61,54 +61,18 @@
     <t xml:space="preserve">% of 2024 Invention Disclosures converted to Filings</t>
   </si>
   <si>
-    <t xml:space="preserve">2024 New Apps Estimate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023 New Apps filed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022 New Apps filed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021 New Apps filed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2020 New Apps filed</t>
-  </si>
-  <si>
     <t xml:space="preserve">Disclosures</t>
   </si>
   <si>
     <t xml:space="preserve">Apps Being Drafted</t>
   </si>
   <si>
-    <t xml:space="preserve">Projects Opened in 2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projects Opened in 2023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projects Opened in 2022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projects Opened in 2021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projects opened in 2020</t>
-  </si>
-  <si>
     <t xml:space="preserve">Total Active Projects</t>
   </si>
   <si>
     <t xml:space="preserve">2022 Issued</t>
   </si>
   <si>
-    <t xml:space="preserve">2024 US Issued</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024 Intl Issued</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Pending Applications</t>
   </si>
   <si>
@@ -149,54 +113,17 @@
   </si>
   <si>
     <t xml:space="preserve">% of Total Portfolio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Update</t>
-  </si>
-  <si>
-    <t xml:space="preserve">03/02/2024</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="SABIC Typeface Headline"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">** </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="SABIC Typeface Headline"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Reductions include both granted &amp; pending applications; includes provisionals (when non-provisonal is not filed), WO-PCTs (if there is no National Stage filing)
-Immediate savings inlcude cost saving resulting from next annuity amount of dropped cases</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">MISC* includes disclosures related to corporate digitilization Program, Local content etc.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EP includes its contracting states patents/applications</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
-    <numFmt numFmtId="166" formatCode="&quot;$ &quot;#,##0,&quot; K&quot;"/>
-    <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -255,38 +182,8 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="SABIC Typeface Headline Light"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="SABIC Typeface Headline Light"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="SABIC Typeface Headline"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -321,12 +218,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFDFEBF7"/>
         <bgColor rgb="FFCCFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -387,173 +278,105 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -808,10 +631,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:DR58"/>
+  <dimension ref="A1:DQ1048576"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.16"/>
@@ -1230,9 +1053,7 @@
       <c r="DQ4" s="6"/>
     </row>
     <row r="5" s="10" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>13</v>
-      </c>
+      <c r="A5" s="7"/>
       <c r="B5" s="8" t="n">
         <v>35</v>
       </c>
@@ -1367,9 +1188,7 @@
       <c r="DQ5" s="6"/>
     </row>
     <row r="6" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
-        <v>14</v>
-      </c>
+      <c r="A6" s="13"/>
       <c r="B6" s="14" t="n">
         <v>43</v>
       </c>
@@ -1401,9 +1220,7 @@
       <c r="P6" s="16"/>
     </row>
     <row r="7" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>15</v>
-      </c>
+      <c r="A7" s="13"/>
       <c r="B7" s="17" t="n">
         <v>41</v>
       </c>
@@ -1433,9 +1250,7 @@
       <c r="P7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
-        <v>16</v>
-      </c>
+      <c r="A8" s="13"/>
       <c r="B8" s="17" t="n">
         <v>25</v>
       </c>
@@ -1465,9 +1280,7 @@
       <c r="P8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
-        <v>17</v>
-      </c>
+      <c r="A9" s="13"/>
       <c r="B9" s="17" t="n">
         <v>30</v>
       </c>
@@ -1502,7 +1315,7 @@
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1522,7 +1335,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -1536,9 +1349,7 @@
       <c r="K11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>20</v>
-      </c>
+      <c r="A12" s="7"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -1551,9 +1362,7 @@
       <c r="K12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>21</v>
-      </c>
+      <c r="A13" s="13"/>
       <c r="B13" s="14" t="n">
         <v>53</v>
       </c>
@@ -1582,9 +1391,7 @@
       <c r="K13" s="4"/>
     </row>
     <row r="14" s="6" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
-        <v>22</v>
-      </c>
+      <c r="A14" s="13"/>
       <c r="B14" s="18" t="n">
         <v>69</v>
       </c>
@@ -1613,9 +1420,7 @@
       <c r="K14" s="4"/>
     </row>
     <row r="15" s="6" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>23</v>
-      </c>
+      <c r="A15" s="13"/>
       <c r="B15" s="18" t="n">
         <v>37</v>
       </c>
@@ -1644,9 +1449,7 @@
       <c r="K15" s="4"/>
     </row>
     <row r="16" s="6" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>24</v>
-      </c>
+      <c r="A16" s="13"/>
       <c r="B16" s="21" t="n">
         <v>50</v>
       </c>
@@ -1676,7 +1479,7 @@
     </row>
     <row r="17" s="6" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>51</v>
@@ -1709,7 +1512,7 @@
     </row>
     <row r="18" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1723,9 +1526,7 @@
       <c r="K18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22" t="s">
-        <v>27</v>
-      </c>
+      <c r="A19" s="22"/>
       <c r="B19" s="23"/>
       <c r="C19" s="23"/>
       <c r="D19" s="23"/>
@@ -1738,9 +1539,7 @@
       <c r="K19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22" t="s">
-        <v>28</v>
-      </c>
+      <c r="A20" s="22"/>
       <c r="B20" s="23"/>
       <c r="C20" s="23"/>
       <c r="D20" s="23"/>
@@ -1754,7 +1553,7 @@
     </row>
     <row r="21" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1769,7 +1568,7 @@
     </row>
     <row r="22" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B22" s="19"/>
       <c r="C22" s="19"/>
@@ -1784,7 +1583,7 @@
     </row>
     <row r="23" s="6" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B23" s="19"/>
       <c r="C23" s="19"/>
@@ -1799,7 +1598,7 @@
     </row>
     <row r="24" s="6" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -1814,7 +1613,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B25" s="19"/>
       <c r="C25" s="19"/>
@@ -1829,7 +1628,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -1844,7 +1643,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1859,7 +1658,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B28" s="19"/>
       <c r="C28" s="19"/>
@@ -1874,7 +1673,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="B29" s="19"/>
       <c r="C29" s="19"/>
@@ -1889,7 +1688,7 @@
     </row>
     <row r="30" s="10" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B30" s="19"/>
       <c r="C30" s="19"/>
@@ -2014,7 +1813,7 @@
     </row>
     <row r="31" s="10" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
@@ -2139,7 +1938,7 @@
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
@@ -2167,7 +1966,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="B34" s="8" t="n">
         <v>471</v>
@@ -2200,7 +1999,7 @@
     </row>
     <row r="35" s="10" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="B35" s="11" t="n">
         <f aca="false">B34/$J$34</f>
@@ -2350,624 +2149,60 @@
       <c r="DP35" s="6"/>
       <c r="DQ35" s="6"/>
     </row>
-    <row r="36" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5"/>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
+    <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0"/>
+      <c r="B36" s="0"/>
+      <c r="C36" s="0"/>
+      <c r="D36" s="0"/>
+      <c r="E36" s="0"/>
+      <c r="F36" s="0"/>
+      <c r="G36" s="0"/>
+      <c r="H36" s="0"/>
+      <c r="I36" s="0"/>
+      <c r="J36" s="0"/>
       <c r="K36" s="4"/>
-      <c r="L36" s="1"/>
-      <c r="M36" s="1"/>
-      <c r="N36" s="1"/>
-      <c r="O36" s="6"/>
-      <c r="P36" s="6"/>
-      <c r="Q36" s="6"/>
-      <c r="R36" s="6"/>
-      <c r="S36" s="6"/>
-      <c r="T36" s="6"/>
-      <c r="U36" s="6"/>
-      <c r="V36" s="6"/>
-      <c r="W36" s="6"/>
-      <c r="X36" s="6"/>
-      <c r="Y36" s="6"/>
-      <c r="Z36" s="6"/>
-      <c r="AA36" s="6"/>
-      <c r="AB36" s="6"/>
-      <c r="AC36" s="6"/>
-      <c r="AD36" s="6"/>
-      <c r="AE36" s="6"/>
-      <c r="AF36" s="6"/>
-      <c r="AG36" s="6"/>
-      <c r="AH36" s="6"/>
-      <c r="AI36" s="6"/>
-      <c r="AJ36" s="6"/>
-      <c r="AK36" s="6"/>
-      <c r="AL36" s="6"/>
-      <c r="AM36" s="6"/>
-      <c r="AN36" s="6"/>
-      <c r="AO36" s="6"/>
-      <c r="AP36" s="6"/>
-      <c r="AQ36" s="6"/>
-      <c r="AR36" s="6"/>
-      <c r="AS36" s="6"/>
-      <c r="AT36" s="6"/>
-      <c r="AU36" s="6"/>
-      <c r="AV36" s="6"/>
-      <c r="AW36" s="6"/>
-      <c r="AX36" s="6"/>
-      <c r="AY36" s="6"/>
-      <c r="AZ36" s="6"/>
-      <c r="BA36" s="6"/>
-      <c r="BB36" s="6"/>
-      <c r="BC36" s="6"/>
-      <c r="BD36" s="6"/>
-      <c r="BE36" s="6"/>
-      <c r="BF36" s="6"/>
-      <c r="BG36" s="6"/>
-      <c r="BH36" s="6"/>
-      <c r="BI36" s="6"/>
-      <c r="BJ36" s="6"/>
-      <c r="BK36" s="6"/>
-      <c r="BL36" s="6"/>
-      <c r="BM36" s="6"/>
-      <c r="BN36" s="6"/>
-      <c r="BO36" s="6"/>
-      <c r="BP36" s="6"/>
-      <c r="BQ36" s="6"/>
-      <c r="BR36" s="6"/>
-      <c r="BS36" s="6"/>
-      <c r="BT36" s="6"/>
-      <c r="BU36" s="6"/>
-      <c r="BV36" s="6"/>
-      <c r="BW36" s="6"/>
-      <c r="BX36" s="6"/>
-      <c r="BY36" s="6"/>
-      <c r="BZ36" s="6"/>
-      <c r="CA36" s="6"/>
-      <c r="CB36" s="6"/>
-      <c r="CC36" s="6"/>
-      <c r="CD36" s="6"/>
-      <c r="CE36" s="6"/>
-      <c r="CF36" s="6"/>
-      <c r="CG36" s="6"/>
-      <c r="CH36" s="6"/>
-      <c r="CI36" s="6"/>
-      <c r="CJ36" s="6"/>
-      <c r="CK36" s="6"/>
-      <c r="CL36" s="6"/>
-      <c r="CM36" s="6"/>
-      <c r="CN36" s="6"/>
-      <c r="CO36" s="6"/>
-      <c r="CP36" s="6"/>
-      <c r="CQ36" s="6"/>
-      <c r="CR36" s="6"/>
-      <c r="CS36" s="6"/>
-      <c r="CT36" s="6"/>
-      <c r="CU36" s="6"/>
-      <c r="CV36" s="6"/>
-      <c r="CW36" s="6"/>
-      <c r="CX36" s="6"/>
-      <c r="CY36" s="6"/>
-      <c r="CZ36" s="6"/>
-      <c r="DA36" s="6"/>
-      <c r="DB36" s="6"/>
-      <c r="DC36" s="6"/>
-      <c r="DD36" s="6"/>
-      <c r="DE36" s="6"/>
-      <c r="DF36" s="6"/>
-      <c r="DG36" s="6"/>
-      <c r="DH36" s="6"/>
-      <c r="DI36" s="6"/>
-      <c r="DJ36" s="6"/>
-      <c r="DK36" s="6"/>
-      <c r="DL36" s="6"/>
-      <c r="DM36" s="6"/>
-      <c r="DN36" s="6"/>
-      <c r="DO36" s="6"/>
-      <c r="DP36" s="6"/>
-      <c r="DQ36" s="6"/>
-      <c r="DR36" s="6"/>
-    </row>
-    <row r="37" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7"/>
-      <c r="B37" s="25"/>
-      <c r="C37" s="25"/>
-      <c r="D37" s="25"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
-      <c r="G37" s="25"/>
-      <c r="H37" s="25"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="26"/>
+    </row>
+    <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
       <c r="K37" s="4"/>
-      <c r="L37" s="27"/>
-      <c r="M37" s="27"/>
-      <c r="N37" s="1"/>
-      <c r="O37" s="6"/>
-      <c r="P37" s="6"/>
-      <c r="Q37" s="6"/>
-      <c r="R37" s="6"/>
-      <c r="S37" s="6"/>
-      <c r="T37" s="6"/>
-      <c r="U37" s="6"/>
-      <c r="V37" s="6"/>
-      <c r="W37" s="6"/>
-      <c r="X37" s="6"/>
-      <c r="Y37" s="6"/>
-      <c r="Z37" s="6"/>
-      <c r="AA37" s="6"/>
-      <c r="AB37" s="6"/>
-      <c r="AC37" s="6"/>
-      <c r="AD37" s="6"/>
-      <c r="AE37" s="6"/>
-      <c r="AF37" s="6"/>
-      <c r="AG37" s="6"/>
-      <c r="AH37" s="6"/>
-      <c r="AI37" s="6"/>
-      <c r="AJ37" s="6"/>
-      <c r="AK37" s="6"/>
-      <c r="AL37" s="6"/>
-      <c r="AM37" s="6"/>
-      <c r="AN37" s="6"/>
-      <c r="AO37" s="6"/>
-      <c r="AP37" s="6"/>
-      <c r="AQ37" s="6"/>
-      <c r="AR37" s="6"/>
-      <c r="AS37" s="6"/>
-      <c r="AT37" s="6"/>
-      <c r="AU37" s="6"/>
-      <c r="AV37" s="6"/>
-      <c r="AW37" s="6"/>
-      <c r="AX37" s="6"/>
-      <c r="AY37" s="6"/>
-      <c r="AZ37" s="6"/>
-      <c r="BA37" s="6"/>
-      <c r="BB37" s="6"/>
-      <c r="BC37" s="6"/>
-      <c r="BD37" s="6"/>
-      <c r="BE37" s="6"/>
-      <c r="BF37" s="6"/>
-      <c r="BG37" s="6"/>
-      <c r="BH37" s="6"/>
-      <c r="BI37" s="6"/>
-      <c r="BJ37" s="6"/>
-      <c r="BK37" s="6"/>
-      <c r="BL37" s="6"/>
-      <c r="BM37" s="6"/>
-      <c r="BN37" s="6"/>
-      <c r="BO37" s="6"/>
-      <c r="BP37" s="6"/>
-      <c r="BQ37" s="6"/>
-      <c r="BR37" s="6"/>
-      <c r="BS37" s="6"/>
-      <c r="BT37" s="6"/>
-      <c r="BU37" s="6"/>
-      <c r="BV37" s="6"/>
-      <c r="BW37" s="6"/>
-      <c r="BX37" s="6"/>
-      <c r="BY37" s="6"/>
-      <c r="BZ37" s="6"/>
-      <c r="CA37" s="6"/>
-      <c r="CB37" s="6"/>
-      <c r="CC37" s="6"/>
-      <c r="CD37" s="6"/>
-      <c r="CE37" s="6"/>
-      <c r="CF37" s="6"/>
-      <c r="CG37" s="6"/>
-      <c r="CH37" s="6"/>
-      <c r="CI37" s="6"/>
-      <c r="CJ37" s="6"/>
-      <c r="CK37" s="6"/>
-      <c r="CL37" s="6"/>
-      <c r="CM37" s="6"/>
-      <c r="CN37" s="6"/>
-      <c r="CO37" s="6"/>
-      <c r="CP37" s="6"/>
-      <c r="CQ37" s="6"/>
-      <c r="CR37" s="6"/>
-      <c r="CS37" s="6"/>
-      <c r="CT37" s="6"/>
-      <c r="CU37" s="6"/>
-      <c r="CV37" s="6"/>
-      <c r="CW37" s="6"/>
-      <c r="CX37" s="6"/>
-      <c r="CY37" s="6"/>
-      <c r="CZ37" s="6"/>
-      <c r="DA37" s="6"/>
-      <c r="DB37" s="6"/>
-      <c r="DC37" s="6"/>
-      <c r="DD37" s="6"/>
-      <c r="DE37" s="6"/>
-      <c r="DF37" s="6"/>
-      <c r="DG37" s="6"/>
-      <c r="DH37" s="6"/>
-      <c r="DI37" s="6"/>
-      <c r="DJ37" s="6"/>
-      <c r="DK37" s="6"/>
-      <c r="DL37" s="6"/>
-      <c r="DM37" s="6"/>
-      <c r="DN37" s="6"/>
-      <c r="DO37" s="6"/>
-      <c r="DP37" s="6"/>
-      <c r="DQ37" s="6"/>
-      <c r="DR37" s="6"/>
-    </row>
-    <row r="38" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
-      <c r="I38" s="5"/>
-      <c r="J38" s="5"/>
-      <c r="K38" s="4"/>
-      <c r="L38" s="1"/>
-      <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
-      <c r="O38" s="6"/>
-      <c r="P38" s="6"/>
-      <c r="Q38" s="6"/>
-      <c r="R38" s="6"/>
-      <c r="S38" s="6"/>
-      <c r="T38" s="6"/>
-      <c r="U38" s="6"/>
-      <c r="V38" s="6"/>
-      <c r="W38" s="6"/>
-      <c r="X38" s="6"/>
-      <c r="Y38" s="6"/>
-      <c r="Z38" s="6"/>
-      <c r="AA38" s="6"/>
-      <c r="AB38" s="6"/>
-      <c r="AC38" s="6"/>
-      <c r="AD38" s="6"/>
-      <c r="AE38" s="6"/>
-      <c r="AF38" s="6"/>
-      <c r="AG38" s="6"/>
-      <c r="AH38" s="6"/>
-      <c r="AI38" s="6"/>
-      <c r="AJ38" s="6"/>
-      <c r="AK38" s="6"/>
-      <c r="AL38" s="6"/>
-      <c r="AM38" s="6"/>
-      <c r="AN38" s="6"/>
-      <c r="AO38" s="6"/>
-      <c r="AP38" s="6"/>
-      <c r="AQ38" s="6"/>
-      <c r="AR38" s="6"/>
-      <c r="AS38" s="6"/>
-      <c r="AT38" s="6"/>
-      <c r="AU38" s="6"/>
-      <c r="AV38" s="6"/>
-      <c r="AW38" s="6"/>
-      <c r="AX38" s="6"/>
-      <c r="AY38" s="6"/>
-      <c r="AZ38" s="6"/>
-      <c r="BA38" s="6"/>
-      <c r="BB38" s="6"/>
-      <c r="BC38" s="6"/>
-      <c r="BD38" s="6"/>
-      <c r="BE38" s="6"/>
-      <c r="BF38" s="6"/>
-      <c r="BG38" s="6"/>
-      <c r="BH38" s="6"/>
-      <c r="BI38" s="6"/>
-      <c r="BJ38" s="6"/>
-      <c r="BK38" s="6"/>
-      <c r="BL38" s="6"/>
-      <c r="BM38" s="6"/>
-      <c r="BN38" s="6"/>
-      <c r="BO38" s="6"/>
-      <c r="BP38" s="6"/>
-      <c r="BQ38" s="6"/>
-      <c r="BR38" s="6"/>
-      <c r="BS38" s="6"/>
-      <c r="BT38" s="6"/>
-      <c r="BU38" s="6"/>
-      <c r="BV38" s="6"/>
-      <c r="BW38" s="6"/>
-      <c r="BX38" s="6"/>
-      <c r="BY38" s="6"/>
-      <c r="BZ38" s="6"/>
-      <c r="CA38" s="6"/>
-      <c r="CB38" s="6"/>
-      <c r="CC38" s="6"/>
-      <c r="CD38" s="6"/>
-      <c r="CE38" s="6"/>
-      <c r="CF38" s="6"/>
-      <c r="CG38" s="6"/>
-      <c r="CH38" s="6"/>
-      <c r="CI38" s="6"/>
-      <c r="CJ38" s="6"/>
-      <c r="CK38" s="6"/>
-      <c r="CL38" s="6"/>
-      <c r="CM38" s="6"/>
-      <c r="CN38" s="6"/>
-      <c r="CO38" s="6"/>
-      <c r="CP38" s="6"/>
-      <c r="CQ38" s="6"/>
-      <c r="CR38" s="6"/>
-      <c r="CS38" s="6"/>
-      <c r="CT38" s="6"/>
-      <c r="CU38" s="6"/>
-      <c r="CV38" s="6"/>
-      <c r="CW38" s="6"/>
-      <c r="CX38" s="6"/>
-      <c r="CY38" s="6"/>
-      <c r="CZ38" s="6"/>
-      <c r="DA38" s="6"/>
-      <c r="DB38" s="6"/>
-      <c r="DC38" s="6"/>
-      <c r="DD38" s="6"/>
-      <c r="DE38" s="6"/>
-      <c r="DF38" s="6"/>
-      <c r="DG38" s="6"/>
-      <c r="DH38" s="6"/>
-      <c r="DI38" s="6"/>
-      <c r="DJ38" s="6"/>
-      <c r="DK38" s="6"/>
-      <c r="DL38" s="6"/>
-      <c r="DM38" s="6"/>
-      <c r="DN38" s="6"/>
-      <c r="DO38" s="6"/>
-      <c r="DP38" s="6"/>
-      <c r="DQ38" s="6"/>
-      <c r="DR38" s="6"/>
-    </row>
-    <row r="39" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="28"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="8"/>
-      <c r="I39" s="9"/>
-      <c r="J39" s="9"/>
-      <c r="K39" s="4"/>
-    </row>
-    <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="29"/>
-      <c r="B40" s="30"/>
-      <c r="C40" s="30"/>
-      <c r="D40" s="31"/>
-      <c r="E40" s="30"/>
-      <c r="F40" s="30"/>
-      <c r="G40" s="30"/>
-      <c r="H40" s="30"/>
-      <c r="I40" s="32"/>
-      <c r="J40" s="32"/>
-      <c r="K40" s="4"/>
-    </row>
-    <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="29"/>
-      <c r="B41" s="30"/>
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
-      <c r="E41" s="30"/>
-      <c r="F41" s="30"/>
-      <c r="G41" s="30"/>
-      <c r="H41" s="30"/>
-      <c r="I41" s="32"/>
-      <c r="J41" s="32"/>
-      <c r="K41" s="4"/>
-    </row>
-    <row r="42" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7"/>
-      <c r="B42" s="25"/>
-      <c r="C42" s="25"/>
-      <c r="D42" s="25"/>
-      <c r="E42" s="25"/>
-      <c r="F42" s="25"/>
-      <c r="G42" s="25"/>
-      <c r="H42" s="25"/>
-      <c r="I42" s="25"/>
-      <c r="J42" s="25"/>
-      <c r="K42" s="4"/>
-    </row>
-    <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="33"/>
-      <c r="B43" s="34"/>
-      <c r="C43" s="34"/>
-      <c r="D43" s="34"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="34"/>
-      <c r="H43" s="35"/>
-      <c r="I43" s="35"/>
-      <c r="J43" s="35"/>
-      <c r="K43" s="4"/>
-    </row>
-    <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="28"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
-      <c r="G44" s="8"/>
-      <c r="H44" s="8"/>
-      <c r="I44" s="9"/>
-      <c r="J44" s="9"/>
-      <c r="K44" s="4"/>
-    </row>
-    <row r="45" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7"/>
-      <c r="B45" s="25"/>
-      <c r="C45" s="25"/>
-      <c r="D45" s="25"/>
-      <c r="E45" s="25"/>
-      <c r="F45" s="25"/>
-      <c r="G45" s="25"/>
-      <c r="H45" s="25"/>
-      <c r="I45" s="26"/>
-      <c r="J45" s="25"/>
-      <c r="K45" s="4"/>
-    </row>
-    <row r="46" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="33"/>
-      <c r="B46" s="34"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="34"/>
-      <c r="H46" s="35"/>
-      <c r="I46" s="35"/>
-      <c r="J46" s="35"/>
-      <c r="K46" s="4"/>
-    </row>
-    <row r="47" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="36"/>
-      <c r="B47" s="25"/>
-      <c r="C47" s="25"/>
-      <c r="D47" s="25"/>
-      <c r="E47" s="25"/>
-      <c r="F47" s="25"/>
-      <c r="G47" s="25"/>
-      <c r="H47" s="25"/>
-      <c r="I47" s="25"/>
-      <c r="J47" s="25"/>
-      <c r="K47" s="4"/>
-    </row>
-    <row r="48" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="33"/>
-      <c r="B48" s="34"/>
-      <c r="C48" s="34"/>
-      <c r="D48" s="34"/>
-      <c r="E48" s="34"/>
-      <c r="F48" s="34"/>
-      <c r="G48" s="34"/>
-      <c r="H48" s="35"/>
-      <c r="I48" s="35"/>
-      <c r="J48" s="35"/>
-      <c r="K48" s="4"/>
-    </row>
-    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="29"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="14"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="15"/>
-      <c r="J49" s="15"/>
-      <c r="K49" s="4"/>
-    </row>
-    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="29"/>
-      <c r="B50" s="30"/>
-      <c r="C50" s="30"/>
-      <c r="D50" s="30"/>
-      <c r="E50" s="30"/>
-      <c r="F50" s="30"/>
-      <c r="G50" s="30"/>
-      <c r="H50" s="30"/>
-      <c r="I50" s="32"/>
-      <c r="J50" s="32"/>
-      <c r="K50" s="4"/>
-    </row>
-    <row r="51" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="37"/>
-      <c r="B51" s="25"/>
-      <c r="C51" s="25"/>
-      <c r="D51" s="25"/>
-      <c r="E51" s="25"/>
-      <c r="F51" s="25"/>
-      <c r="G51" s="25"/>
-      <c r="H51" s="25"/>
-      <c r="I51" s="25"/>
-      <c r="J51" s="25"/>
-      <c r="K51" s="4"/>
-    </row>
-    <row r="52" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K52" s="4"/>
-    </row>
-    <row r="53" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="38" t="s">
-        <v>43</v>
-      </c>
-      <c r="B53" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="E53" s="35"/>
-      <c r="F53" s="6"/>
-      <c r="K53" s="4"/>
-    </row>
-    <row r="54" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="40"/>
-      <c r="K54" s="4"/>
-    </row>
-    <row r="55" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="41" t="s">
-        <v>45</v>
-      </c>
-      <c r="B55" s="41"/>
-      <c r="C55" s="41"/>
-      <c r="D55" s="41"/>
-      <c r="E55" s="41"/>
-      <c r="F55" s="41"/>
-      <c r="G55" s="41"/>
-      <c r="H55" s="41"/>
-      <c r="I55" s="41"/>
-      <c r="J55" s="41"/>
-      <c r="K55" s="4"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B56" s="33"/>
-      <c r="C56" s="33"/>
-      <c r="D56" s="33"/>
-      <c r="E56" s="33"/>
-      <c r="F56" s="33"/>
-      <c r="G56" s="33"/>
-      <c r="H56" s="33"/>
-      <c r="I56" s="33"/>
-      <c r="J56" s="33"/>
-      <c r="K56" s="4"/>
-    </row>
-    <row r="57" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="33" t="s">
-        <v>47</v>
-      </c>
-      <c r="K57" s="4"/>
-    </row>
-    <row r="58" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="4"/>
-      <c r="B58" s="4"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4"/>
-    </row>
+    </row>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="5">
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A10:J10"/>
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="A21:J21"/>
     <mergeCell ref="A27:J27"/>
-    <mergeCell ref="A36:J36"/>
-    <mergeCell ref="A38:J38"/>
-    <mergeCell ref="A55:J55"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
monthly ip in progress with new sop
</commit_message>
<xml_diff>
--- a/reports/sample/sample-monthly-ip-report.xlsx
+++ b/reports/sample/sample-monthly-ip-report.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t xml:space="preserve">SBU</t>
   </si>
@@ -104,6 +104,9 @@
   </si>
   <si>
     <t xml:space="preserve">% of Total Portfolio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reductions &amp; Cost Savings</t>
   </si>
 </sst>
 </file>
@@ -277,7 +280,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -382,6 +385,18 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -398,20 +413,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2020,268 +2031,405 @@
       <c r="K35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="26"/>
-      <c r="B36" s="26"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="26"/>
-      <c r="J36" s="26"/>
-      <c r="K36" s="27"/>
-      <c r="L36" s="28"/>
-      <c r="M36" s="28"/>
-      <c r="N36" s="28"/>
-      <c r="O36" s="29"/>
-      <c r="P36" s="29"/>
-      <c r="Q36" s="29"/>
-      <c r="R36" s="29"/>
-      <c r="S36" s="29"/>
-      <c r="T36" s="29"/>
-      <c r="U36" s="29"/>
-      <c r="V36" s="29"/>
-      <c r="W36" s="29"/>
-      <c r="X36" s="29"/>
-      <c r="Y36" s="29"/>
-      <c r="Z36" s="29"/>
-      <c r="AA36" s="29"/>
-      <c r="AB36" s="29"/>
-      <c r="AC36" s="29"/>
-      <c r="AD36" s="29"/>
-      <c r="AE36" s="29"/>
-      <c r="AF36" s="29"/>
-      <c r="AG36" s="29"/>
-      <c r="AH36" s="29"/>
-      <c r="AI36" s="29"/>
-      <c r="AJ36" s="29"/>
-      <c r="AK36" s="29"/>
-      <c r="AL36" s="29"/>
-      <c r="AM36" s="29"/>
-      <c r="AN36" s="29"/>
-      <c r="AO36" s="29"/>
-      <c r="AP36" s="29"/>
-      <c r="AQ36" s="29"/>
-      <c r="AR36" s="29"/>
-      <c r="AS36" s="29"/>
-      <c r="AT36" s="29"/>
-      <c r="AU36" s="29"/>
-      <c r="AV36" s="29"/>
-      <c r="AW36" s="29"/>
-      <c r="AX36" s="29"/>
-      <c r="AY36" s="29"/>
-      <c r="AZ36" s="29"/>
-      <c r="BA36" s="29"/>
-      <c r="BB36" s="29"/>
-      <c r="BC36" s="29"/>
-      <c r="BD36" s="29"/>
-      <c r="BE36" s="29"/>
-      <c r="BF36" s="29"/>
-      <c r="BG36" s="29"/>
-      <c r="BH36" s="29"/>
-      <c r="BI36" s="29"/>
-      <c r="BJ36" s="29"/>
-      <c r="BK36" s="29"/>
-      <c r="BL36" s="29"/>
-      <c r="BM36" s="29"/>
-      <c r="BN36" s="29"/>
-      <c r="BO36" s="29"/>
-      <c r="BP36" s="29"/>
-      <c r="BQ36" s="29"/>
-      <c r="BR36" s="29"/>
-      <c r="BS36" s="29"/>
-      <c r="BT36" s="29"/>
-      <c r="BU36" s="29"/>
-      <c r="BV36" s="29"/>
-      <c r="BW36" s="29"/>
-      <c r="BX36" s="29"/>
-      <c r="BY36" s="29"/>
-      <c r="BZ36" s="29"/>
-      <c r="CA36" s="29"/>
-      <c r="CB36" s="29"/>
-      <c r="CC36" s="29"/>
-      <c r="CD36" s="29"/>
-      <c r="CE36" s="29"/>
-      <c r="CF36" s="29"/>
-      <c r="CG36" s="29"/>
-      <c r="CH36" s="29"/>
-      <c r="CI36" s="29"/>
-      <c r="CJ36" s="29"/>
-      <c r="CK36" s="29"/>
-      <c r="CL36" s="29"/>
-      <c r="CM36" s="29"/>
-      <c r="CN36" s="29"/>
-      <c r="CO36" s="29"/>
-      <c r="CP36" s="29"/>
-      <c r="CQ36" s="29"/>
-      <c r="CR36" s="29"/>
-      <c r="CS36" s="29"/>
-      <c r="CT36" s="29"/>
-      <c r="CU36" s="29"/>
-      <c r="CV36" s="29"/>
-      <c r="CW36" s="29"/>
-      <c r="CX36" s="29"/>
-      <c r="CY36" s="29"/>
-      <c r="CZ36" s="29"/>
-      <c r="DA36" s="29"/>
-      <c r="DB36" s="29"/>
-      <c r="DC36" s="29"/>
-      <c r="DD36" s="29"/>
-      <c r="DE36" s="29"/>
-      <c r="DF36" s="29"/>
-      <c r="DG36" s="29"/>
-      <c r="DH36" s="29"/>
-      <c r="DI36" s="29"/>
-      <c r="DJ36" s="29"/>
-      <c r="DK36" s="29"/>
-      <c r="DL36" s="29"/>
-      <c r="DM36" s="29"/>
-      <c r="DN36" s="29"/>
-      <c r="DO36" s="29"/>
-      <c r="DP36" s="29"/>
-      <c r="DQ36" s="29"/>
-      <c r="DR36" s="29"/>
+      <c r="A36" s="6"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="6"/>
+      <c r="K36" s="5"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+      <c r="O36" s="7"/>
+      <c r="P36" s="7"/>
+      <c r="Q36" s="7"/>
+      <c r="R36" s="7"/>
+      <c r="S36" s="7"/>
+      <c r="T36" s="7"/>
+      <c r="U36" s="7"/>
+      <c r="V36" s="7"/>
+      <c r="W36" s="7"/>
+      <c r="X36" s="7"/>
+      <c r="Y36" s="7"/>
+      <c r="Z36" s="7"/>
+      <c r="AA36" s="7"/>
+      <c r="AB36" s="7"/>
+      <c r="AC36" s="7"/>
+      <c r="AD36" s="7"/>
+      <c r="AE36" s="7"/>
+      <c r="AF36" s="7"/>
+      <c r="AG36" s="7"/>
+      <c r="AH36" s="7"/>
+      <c r="AI36" s="7"/>
+      <c r="AJ36" s="7"/>
+      <c r="AK36" s="7"/>
+      <c r="AL36" s="7"/>
+      <c r="AM36" s="7"/>
+      <c r="AN36" s="7"/>
+      <c r="AO36" s="7"/>
+      <c r="AP36" s="7"/>
+      <c r="AQ36" s="7"/>
+      <c r="AR36" s="7"/>
+      <c r="AS36" s="7"/>
+      <c r="AT36" s="7"/>
+      <c r="AU36" s="7"/>
+      <c r="AV36" s="7"/>
+      <c r="AW36" s="7"/>
+      <c r="AX36" s="7"/>
+      <c r="AY36" s="7"/>
+      <c r="AZ36" s="7"/>
+      <c r="BA36" s="7"/>
+      <c r="BB36" s="7"/>
+      <c r="BC36" s="7"/>
+      <c r="BD36" s="7"/>
+      <c r="BE36" s="7"/>
+      <c r="BF36" s="7"/>
+      <c r="BG36" s="7"/>
+      <c r="BH36" s="7"/>
+      <c r="BI36" s="7"/>
+      <c r="BJ36" s="7"/>
+      <c r="BK36" s="7"/>
+      <c r="BL36" s="7"/>
+      <c r="BM36" s="7"/>
+      <c r="BN36" s="7"/>
+      <c r="BO36" s="7"/>
+      <c r="BP36" s="7"/>
+      <c r="BQ36" s="7"/>
+      <c r="BR36" s="7"/>
+      <c r="BS36" s="7"/>
+      <c r="BT36" s="7"/>
+      <c r="BU36" s="7"/>
+      <c r="BV36" s="7"/>
+      <c r="BW36" s="7"/>
+      <c r="BX36" s="7"/>
+      <c r="BY36" s="7"/>
+      <c r="BZ36" s="7"/>
+      <c r="CA36" s="7"/>
+      <c r="CB36" s="7"/>
+      <c r="CC36" s="7"/>
+      <c r="CD36" s="7"/>
+      <c r="CE36" s="7"/>
+      <c r="CF36" s="7"/>
+      <c r="CG36" s="7"/>
+      <c r="CH36" s="7"/>
+      <c r="CI36" s="7"/>
+      <c r="CJ36" s="7"/>
+      <c r="CK36" s="7"/>
+      <c r="CL36" s="7"/>
+      <c r="CM36" s="7"/>
+      <c r="CN36" s="7"/>
+      <c r="CO36" s="7"/>
+      <c r="CP36" s="7"/>
+      <c r="CQ36" s="7"/>
+      <c r="CR36" s="7"/>
+      <c r="CS36" s="7"/>
+      <c r="CT36" s="7"/>
+      <c r="CU36" s="7"/>
+      <c r="CV36" s="7"/>
+      <c r="CW36" s="7"/>
+      <c r="CX36" s="7"/>
+      <c r="CY36" s="7"/>
+      <c r="CZ36" s="7"/>
+      <c r="DA36" s="7"/>
+      <c r="DB36" s="7"/>
+      <c r="DC36" s="7"/>
+      <c r="DD36" s="7"/>
+      <c r="DE36" s="7"/>
+      <c r="DF36" s="7"/>
+      <c r="DG36" s="7"/>
+      <c r="DH36" s="7"/>
+      <c r="DI36" s="7"/>
+      <c r="DJ36" s="7"/>
+      <c r="DK36" s="7"/>
+      <c r="DL36" s="7"/>
+      <c r="DM36" s="7"/>
+      <c r="DN36" s="7"/>
+      <c r="DO36" s="7"/>
+      <c r="DP36" s="7"/>
+      <c r="DQ36" s="7"/>
+      <c r="DR36" s="7"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="30"/>
-      <c r="B37" s="31"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="31"/>
-      <c r="F37" s="31"/>
-      <c r="G37" s="31"/>
-      <c r="H37" s="31"/>
-      <c r="I37" s="32"/>
-      <c r="J37" s="32"/>
-      <c r="K37" s="27"/>
-      <c r="L37" s="33"/>
-      <c r="M37" s="33"/>
-      <c r="N37" s="28"/>
-      <c r="O37" s="29"/>
-      <c r="P37" s="29"/>
-      <c r="Q37" s="29"/>
-      <c r="R37" s="29"/>
-      <c r="S37" s="29"/>
-      <c r="T37" s="29"/>
-      <c r="U37" s="29"/>
-      <c r="V37" s="29"/>
-      <c r="W37" s="29"/>
-      <c r="X37" s="29"/>
-      <c r="Y37" s="29"/>
-      <c r="Z37" s="29"/>
-      <c r="AA37" s="29"/>
-      <c r="AB37" s="29"/>
-      <c r="AC37" s="29"/>
-      <c r="AD37" s="29"/>
-      <c r="AE37" s="29"/>
-      <c r="AF37" s="29"/>
-      <c r="AG37" s="29"/>
-      <c r="AH37" s="29"/>
-      <c r="AI37" s="29"/>
-      <c r="AJ37" s="29"/>
-      <c r="AK37" s="29"/>
-      <c r="AL37" s="29"/>
-      <c r="AM37" s="29"/>
-      <c r="AN37" s="29"/>
-      <c r="AO37" s="29"/>
-      <c r="AP37" s="29"/>
-      <c r="AQ37" s="29"/>
-      <c r="AR37" s="29"/>
-      <c r="AS37" s="29"/>
-      <c r="AT37" s="29"/>
-      <c r="AU37" s="29"/>
-      <c r="AV37" s="29"/>
-      <c r="AW37" s="29"/>
-      <c r="AX37" s="29"/>
-      <c r="AY37" s="29"/>
-      <c r="AZ37" s="29"/>
-      <c r="BA37" s="29"/>
-      <c r="BB37" s="29"/>
-      <c r="BC37" s="29"/>
-      <c r="BD37" s="29"/>
-      <c r="BE37" s="29"/>
-      <c r="BF37" s="29"/>
-      <c r="BG37" s="29"/>
-      <c r="BH37" s="29"/>
-      <c r="BI37" s="29"/>
-      <c r="BJ37" s="29"/>
-      <c r="BK37" s="29"/>
-      <c r="BL37" s="29"/>
-      <c r="BM37" s="29"/>
-      <c r="BN37" s="29"/>
-      <c r="BO37" s="29"/>
-      <c r="BP37" s="29"/>
-      <c r="BQ37" s="29"/>
-      <c r="BR37" s="29"/>
-      <c r="BS37" s="29"/>
-      <c r="BT37" s="29"/>
-      <c r="BU37" s="29"/>
-      <c r="BV37" s="29"/>
-      <c r="BW37" s="29"/>
-      <c r="BX37" s="29"/>
-      <c r="BY37" s="29"/>
-      <c r="BZ37" s="29"/>
-      <c r="CA37" s="29"/>
-      <c r="CB37" s="29"/>
-      <c r="CC37" s="29"/>
-      <c r="CD37" s="29"/>
-      <c r="CE37" s="29"/>
-      <c r="CF37" s="29"/>
-      <c r="CG37" s="29"/>
-      <c r="CH37" s="29"/>
-      <c r="CI37" s="29"/>
-      <c r="CJ37" s="29"/>
-      <c r="CK37" s="29"/>
-      <c r="CL37" s="29"/>
-      <c r="CM37" s="29"/>
-      <c r="CN37" s="29"/>
-      <c r="CO37" s="29"/>
-      <c r="CP37" s="29"/>
-      <c r="CQ37" s="29"/>
-      <c r="CR37" s="29"/>
-      <c r="CS37" s="29"/>
-      <c r="CT37" s="29"/>
-      <c r="CU37" s="29"/>
-      <c r="CV37" s="29"/>
-      <c r="CW37" s="29"/>
-      <c r="CX37" s="29"/>
-      <c r="CY37" s="29"/>
-      <c r="CZ37" s="29"/>
-      <c r="DA37" s="29"/>
-      <c r="DB37" s="29"/>
-      <c r="DC37" s="29"/>
-      <c r="DD37" s="29"/>
-      <c r="DE37" s="29"/>
-      <c r="DF37" s="29"/>
-      <c r="DG37" s="29"/>
-      <c r="DH37" s="29"/>
-      <c r="DI37" s="29"/>
-      <c r="DJ37" s="29"/>
-      <c r="DK37" s="29"/>
-      <c r="DL37" s="29"/>
-      <c r="DM37" s="29"/>
-      <c r="DN37" s="29"/>
-      <c r="DO37" s="29"/>
-      <c r="DP37" s="29"/>
-      <c r="DQ37" s="29"/>
-      <c r="DR37" s="29"/>
-    </row>
-    <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
-      <c r="I38" s="5"/>
-      <c r="J38" s="5"/>
-      <c r="K38" s="5"/>
-    </row>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A37" s="8"/>
+      <c r="B37" s="26"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="26"/>
+      <c r="F37" s="26"/>
+      <c r="G37" s="26"/>
+      <c r="H37" s="26"/>
+      <c r="I37" s="27"/>
+      <c r="J37" s="27"/>
+      <c r="K37" s="5"/>
+      <c r="L37" s="28"/>
+      <c r="M37" s="28"/>
+      <c r="N37" s="1"/>
+      <c r="O37" s="7"/>
+      <c r="P37" s="7"/>
+      <c r="Q37" s="7"/>
+      <c r="R37" s="7"/>
+      <c r="S37" s="7"/>
+      <c r="T37" s="7"/>
+      <c r="U37" s="7"/>
+      <c r="V37" s="7"/>
+      <c r="W37" s="7"/>
+      <c r="X37" s="7"/>
+      <c r="Y37" s="7"/>
+      <c r="Z37" s="7"/>
+      <c r="AA37" s="7"/>
+      <c r="AB37" s="7"/>
+      <c r="AC37" s="7"/>
+      <c r="AD37" s="7"/>
+      <c r="AE37" s="7"/>
+      <c r="AF37" s="7"/>
+      <c r="AG37" s="7"/>
+      <c r="AH37" s="7"/>
+      <c r="AI37" s="7"/>
+      <c r="AJ37" s="7"/>
+      <c r="AK37" s="7"/>
+      <c r="AL37" s="7"/>
+      <c r="AM37" s="7"/>
+      <c r="AN37" s="7"/>
+      <c r="AO37" s="7"/>
+      <c r="AP37" s="7"/>
+      <c r="AQ37" s="7"/>
+      <c r="AR37" s="7"/>
+      <c r="AS37" s="7"/>
+      <c r="AT37" s="7"/>
+      <c r="AU37" s="7"/>
+      <c r="AV37" s="7"/>
+      <c r="AW37" s="7"/>
+      <c r="AX37" s="7"/>
+      <c r="AY37" s="7"/>
+      <c r="AZ37" s="7"/>
+      <c r="BA37" s="7"/>
+      <c r="BB37" s="7"/>
+      <c r="BC37" s="7"/>
+      <c r="BD37" s="7"/>
+      <c r="BE37" s="7"/>
+      <c r="BF37" s="7"/>
+      <c r="BG37" s="7"/>
+      <c r="BH37" s="7"/>
+      <c r="BI37" s="7"/>
+      <c r="BJ37" s="7"/>
+      <c r="BK37" s="7"/>
+      <c r="BL37" s="7"/>
+      <c r="BM37" s="7"/>
+      <c r="BN37" s="7"/>
+      <c r="BO37" s="7"/>
+      <c r="BP37" s="7"/>
+      <c r="BQ37" s="7"/>
+      <c r="BR37" s="7"/>
+      <c r="BS37" s="7"/>
+      <c r="BT37" s="7"/>
+      <c r="BU37" s="7"/>
+      <c r="BV37" s="7"/>
+      <c r="BW37" s="7"/>
+      <c r="BX37" s="7"/>
+      <c r="BY37" s="7"/>
+      <c r="BZ37" s="7"/>
+      <c r="CA37" s="7"/>
+      <c r="CB37" s="7"/>
+      <c r="CC37" s="7"/>
+      <c r="CD37" s="7"/>
+      <c r="CE37" s="7"/>
+      <c r="CF37" s="7"/>
+      <c r="CG37" s="7"/>
+      <c r="CH37" s="7"/>
+      <c r="CI37" s="7"/>
+      <c r="CJ37" s="7"/>
+      <c r="CK37" s="7"/>
+      <c r="CL37" s="7"/>
+      <c r="CM37" s="7"/>
+      <c r="CN37" s="7"/>
+      <c r="CO37" s="7"/>
+      <c r="CP37" s="7"/>
+      <c r="CQ37" s="7"/>
+      <c r="CR37" s="7"/>
+      <c r="CS37" s="7"/>
+      <c r="CT37" s="7"/>
+      <c r="CU37" s="7"/>
+      <c r="CV37" s="7"/>
+      <c r="CW37" s="7"/>
+      <c r="CX37" s="7"/>
+      <c r="CY37" s="7"/>
+      <c r="CZ37" s="7"/>
+      <c r="DA37" s="7"/>
+      <c r="DB37" s="7"/>
+      <c r="DC37" s="7"/>
+      <c r="DD37" s="7"/>
+      <c r="DE37" s="7"/>
+      <c r="DF37" s="7"/>
+      <c r="DG37" s="7"/>
+      <c r="DH37" s="7"/>
+      <c r="DI37" s="7"/>
+      <c r="DJ37" s="7"/>
+      <c r="DK37" s="7"/>
+      <c r="DL37" s="7"/>
+      <c r="DM37" s="7"/>
+      <c r="DN37" s="7"/>
+      <c r="DO37" s="7"/>
+      <c r="DP37" s="7"/>
+      <c r="DQ37" s="7"/>
+      <c r="DR37" s="7"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="29"/>
+      <c r="J38" s="29"/>
+      <c r="K38" s="30"/>
+      <c r="L38" s="31"/>
+      <c r="M38" s="31"/>
+      <c r="N38" s="31"/>
+      <c r="O38" s="32"/>
+      <c r="P38" s="32"/>
+      <c r="Q38" s="32"/>
+      <c r="R38" s="32"/>
+      <c r="S38" s="32"/>
+      <c r="T38" s="32"/>
+      <c r="U38" s="32"/>
+      <c r="V38" s="32"/>
+      <c r="W38" s="32"/>
+      <c r="X38" s="32"/>
+      <c r="Y38" s="32"/>
+      <c r="Z38" s="32"/>
+      <c r="AA38" s="32"/>
+      <c r="AB38" s="32"/>
+      <c r="AC38" s="32"/>
+      <c r="AD38" s="32"/>
+      <c r="AE38" s="32"/>
+      <c r="AF38" s="32"/>
+      <c r="AG38" s="32"/>
+      <c r="AH38" s="32"/>
+      <c r="AI38" s="32"/>
+      <c r="AJ38" s="32"/>
+      <c r="AK38" s="32"/>
+      <c r="AL38" s="32"/>
+      <c r="AM38" s="32"/>
+      <c r="AN38" s="32"/>
+      <c r="AO38" s="32"/>
+      <c r="AP38" s="32"/>
+      <c r="AQ38" s="32"/>
+      <c r="AR38" s="32"/>
+      <c r="AS38" s="32"/>
+      <c r="AT38" s="32"/>
+      <c r="AU38" s="32"/>
+      <c r="AV38" s="32"/>
+      <c r="AW38" s="32"/>
+      <c r="AX38" s="32"/>
+      <c r="AY38" s="32"/>
+      <c r="AZ38" s="32"/>
+      <c r="BA38" s="32"/>
+      <c r="BB38" s="32"/>
+      <c r="BC38" s="32"/>
+      <c r="BD38" s="32"/>
+      <c r="BE38" s="32"/>
+      <c r="BF38" s="32"/>
+      <c r="BG38" s="32"/>
+      <c r="BH38" s="32"/>
+      <c r="BI38" s="32"/>
+      <c r="BJ38" s="32"/>
+      <c r="BK38" s="32"/>
+      <c r="BL38" s="32"/>
+      <c r="BM38" s="32"/>
+      <c r="BN38" s="32"/>
+      <c r="BO38" s="32"/>
+      <c r="BP38" s="32"/>
+      <c r="BQ38" s="32"/>
+      <c r="BR38" s="32"/>
+      <c r="BS38" s="32"/>
+      <c r="BT38" s="32"/>
+      <c r="BU38" s="32"/>
+      <c r="BV38" s="32"/>
+      <c r="BW38" s="32"/>
+      <c r="BX38" s="32"/>
+      <c r="BY38" s="32"/>
+      <c r="BZ38" s="32"/>
+      <c r="CA38" s="32"/>
+      <c r="CB38" s="32"/>
+      <c r="CC38" s="32"/>
+      <c r="CD38" s="32"/>
+      <c r="CE38" s="32"/>
+      <c r="CF38" s="32"/>
+      <c r="CG38" s="32"/>
+      <c r="CH38" s="32"/>
+      <c r="CI38" s="32"/>
+      <c r="CJ38" s="32"/>
+      <c r="CK38" s="32"/>
+      <c r="CL38" s="32"/>
+      <c r="CM38" s="32"/>
+      <c r="CN38" s="32"/>
+      <c r="CO38" s="32"/>
+      <c r="CP38" s="32"/>
+      <c r="CQ38" s="32"/>
+      <c r="CR38" s="32"/>
+      <c r="CS38" s="32"/>
+      <c r="CT38" s="32"/>
+      <c r="CU38" s="32"/>
+      <c r="CV38" s="32"/>
+      <c r="CW38" s="32"/>
+      <c r="CX38" s="32"/>
+      <c r="CY38" s="32"/>
+      <c r="CZ38" s="32"/>
+      <c r="DA38" s="32"/>
+      <c r="DB38" s="32"/>
+      <c r="DC38" s="32"/>
+      <c r="DD38" s="32"/>
+      <c r="DE38" s="32"/>
+      <c r="DF38" s="32"/>
+      <c r="DG38" s="32"/>
+      <c r="DH38" s="32"/>
+      <c r="DI38" s="32"/>
+      <c r="DJ38" s="32"/>
+      <c r="DK38" s="32"/>
+      <c r="DL38" s="32"/>
+      <c r="DM38" s="32"/>
+      <c r="DN38" s="32"/>
+      <c r="DO38" s="32"/>
+      <c r="DP38" s="32"/>
+      <c r="DQ38" s="32"/>
+      <c r="DR38" s="32"/>
+    </row>
+    <row r="39" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="33"/>
+      <c r="B39" s="34"/>
+      <c r="C39" s="34"/>
+      <c r="D39" s="34"/>
+      <c r="E39" s="34"/>
+      <c r="F39" s="34"/>
+      <c r="G39" s="34"/>
+      <c r="H39" s="34"/>
+      <c r="I39" s="35"/>
+      <c r="J39" s="35"/>
+      <c r="K39" s="30"/>
+      <c r="L39" s="31"/>
+    </row>
+    <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5"/>
+      <c r="K40" s="5"/>
+    </row>
     <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2301,13 +2449,14 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A10:J10"/>
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="A21:J21"/>
     <mergeCell ref="A27:J27"/>
     <mergeCell ref="A36:J36"/>
+    <mergeCell ref="A38:J38"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
update in monthly ip report is in progress
</commit_message>
<xml_diff>
--- a/reports/sample/sample-monthly-ip-report.xlsx
+++ b/reports/sample/sample-monthly-ip-report.xlsx
@@ -113,10 +113,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
     <numFmt numFmtId="166" formatCode="&quot;$ &quot;#,##0,&quot; K&quot;"/>
+    <numFmt numFmtId="167" formatCode="&quot;$ &quot;#,##0,&quot; K&quot;"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -280,7 +281,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -397,20 +398,44 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -423,6 +448,14 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2278,167 +2311,273 @@
       <c r="DR37" s="7"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="29" t="s">
+      <c r="A38" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B38" s="29"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="29"/>
-      <c r="G38" s="29"/>
-      <c r="H38" s="29"/>
-      <c r="I38" s="29"/>
-      <c r="J38" s="29"/>
-      <c r="K38" s="30"/>
-      <c r="L38" s="31"/>
-      <c r="M38" s="31"/>
-      <c r="N38" s="31"/>
-      <c r="O38" s="32"/>
-      <c r="P38" s="32"/>
-      <c r="Q38" s="32"/>
-      <c r="R38" s="32"/>
-      <c r="S38" s="32"/>
-      <c r="T38" s="32"/>
-      <c r="U38" s="32"/>
-      <c r="V38" s="32"/>
-      <c r="W38" s="32"/>
-      <c r="X38" s="32"/>
-      <c r="Y38" s="32"/>
-      <c r="Z38" s="32"/>
-      <c r="AA38" s="32"/>
-      <c r="AB38" s="32"/>
-      <c r="AC38" s="32"/>
-      <c r="AD38" s="32"/>
-      <c r="AE38" s="32"/>
-      <c r="AF38" s="32"/>
-      <c r="AG38" s="32"/>
-      <c r="AH38" s="32"/>
-      <c r="AI38" s="32"/>
-      <c r="AJ38" s="32"/>
-      <c r="AK38" s="32"/>
-      <c r="AL38" s="32"/>
-      <c r="AM38" s="32"/>
-      <c r="AN38" s="32"/>
-      <c r="AO38" s="32"/>
-      <c r="AP38" s="32"/>
-      <c r="AQ38" s="32"/>
-      <c r="AR38" s="32"/>
-      <c r="AS38" s="32"/>
-      <c r="AT38" s="32"/>
-      <c r="AU38" s="32"/>
-      <c r="AV38" s="32"/>
-      <c r="AW38" s="32"/>
-      <c r="AX38" s="32"/>
-      <c r="AY38" s="32"/>
-      <c r="AZ38" s="32"/>
-      <c r="BA38" s="32"/>
-      <c r="BB38" s="32"/>
-      <c r="BC38" s="32"/>
-      <c r="BD38" s="32"/>
-      <c r="BE38" s="32"/>
-      <c r="BF38" s="32"/>
-      <c r="BG38" s="32"/>
-      <c r="BH38" s="32"/>
-      <c r="BI38" s="32"/>
-      <c r="BJ38" s="32"/>
-      <c r="BK38" s="32"/>
-      <c r="BL38" s="32"/>
-      <c r="BM38" s="32"/>
-      <c r="BN38" s="32"/>
-      <c r="BO38" s="32"/>
-      <c r="BP38" s="32"/>
-      <c r="BQ38" s="32"/>
-      <c r="BR38" s="32"/>
-      <c r="BS38" s="32"/>
-      <c r="BT38" s="32"/>
-      <c r="BU38" s="32"/>
-      <c r="BV38" s="32"/>
-      <c r="BW38" s="32"/>
-      <c r="BX38" s="32"/>
-      <c r="BY38" s="32"/>
-      <c r="BZ38" s="32"/>
-      <c r="CA38" s="32"/>
-      <c r="CB38" s="32"/>
-      <c r="CC38" s="32"/>
-      <c r="CD38" s="32"/>
-      <c r="CE38" s="32"/>
-      <c r="CF38" s="32"/>
-      <c r="CG38" s="32"/>
-      <c r="CH38" s="32"/>
-      <c r="CI38" s="32"/>
-      <c r="CJ38" s="32"/>
-      <c r="CK38" s="32"/>
-      <c r="CL38" s="32"/>
-      <c r="CM38" s="32"/>
-      <c r="CN38" s="32"/>
-      <c r="CO38" s="32"/>
-      <c r="CP38" s="32"/>
-      <c r="CQ38" s="32"/>
-      <c r="CR38" s="32"/>
-      <c r="CS38" s="32"/>
-      <c r="CT38" s="32"/>
-      <c r="CU38" s="32"/>
-      <c r="CV38" s="32"/>
-      <c r="CW38" s="32"/>
-      <c r="CX38" s="32"/>
-      <c r="CY38" s="32"/>
-      <c r="CZ38" s="32"/>
-      <c r="DA38" s="32"/>
-      <c r="DB38" s="32"/>
-      <c r="DC38" s="32"/>
-      <c r="DD38" s="32"/>
-      <c r="DE38" s="32"/>
-      <c r="DF38" s="32"/>
-      <c r="DG38" s="32"/>
-      <c r="DH38" s="32"/>
-      <c r="DI38" s="32"/>
-      <c r="DJ38" s="32"/>
-      <c r="DK38" s="32"/>
-      <c r="DL38" s="32"/>
-      <c r="DM38" s="32"/>
-      <c r="DN38" s="32"/>
-      <c r="DO38" s="32"/>
-      <c r="DP38" s="32"/>
-      <c r="DQ38" s="32"/>
-      <c r="DR38" s="32"/>
-    </row>
-    <row r="39" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="33"/>
-      <c r="B39" s="34"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="34"/>
-      <c r="E39" s="34"/>
-      <c r="F39" s="34"/>
-      <c r="G39" s="34"/>
-      <c r="H39" s="34"/>
-      <c r="I39" s="35"/>
-      <c r="J39" s="35"/>
-      <c r="K39" s="30"/>
-      <c r="L39" s="31"/>
-    </row>
-    <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="5"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="6"/>
+      <c r="J38" s="6"/>
+      <c r="K38" s="5"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1"/>
+      <c r="O38" s="7"/>
+      <c r="P38" s="7"/>
+      <c r="Q38" s="7"/>
+      <c r="R38" s="7"/>
+      <c r="S38" s="7"/>
+      <c r="T38" s="7"/>
+      <c r="U38" s="7"/>
+      <c r="V38" s="7"/>
+      <c r="W38" s="7"/>
+      <c r="X38" s="7"/>
+      <c r="Y38" s="7"/>
+      <c r="Z38" s="7"/>
+      <c r="AA38" s="7"/>
+      <c r="AB38" s="7"/>
+      <c r="AC38" s="7"/>
+      <c r="AD38" s="7"/>
+      <c r="AE38" s="7"/>
+      <c r="AF38" s="7"/>
+      <c r="AG38" s="7"/>
+      <c r="AH38" s="7"/>
+      <c r="AI38" s="7"/>
+      <c r="AJ38" s="7"/>
+      <c r="AK38" s="7"/>
+      <c r="AL38" s="7"/>
+      <c r="AM38" s="7"/>
+      <c r="AN38" s="7"/>
+      <c r="AO38" s="7"/>
+      <c r="AP38" s="7"/>
+      <c r="AQ38" s="7"/>
+      <c r="AR38" s="7"/>
+      <c r="AS38" s="7"/>
+      <c r="AT38" s="7"/>
+      <c r="AU38" s="7"/>
+      <c r="AV38" s="7"/>
+      <c r="AW38" s="7"/>
+      <c r="AX38" s="7"/>
+      <c r="AY38" s="7"/>
+      <c r="AZ38" s="7"/>
+      <c r="BA38" s="7"/>
+      <c r="BB38" s="7"/>
+      <c r="BC38" s="7"/>
+      <c r="BD38" s="7"/>
+      <c r="BE38" s="7"/>
+      <c r="BF38" s="7"/>
+      <c r="BG38" s="7"/>
+      <c r="BH38" s="7"/>
+      <c r="BI38" s="7"/>
+      <c r="BJ38" s="7"/>
+      <c r="BK38" s="7"/>
+      <c r="BL38" s="7"/>
+      <c r="BM38" s="7"/>
+      <c r="BN38" s="7"/>
+      <c r="BO38" s="7"/>
+      <c r="BP38" s="7"/>
+      <c r="BQ38" s="7"/>
+      <c r="BR38" s="7"/>
+      <c r="BS38" s="7"/>
+      <c r="BT38" s="7"/>
+      <c r="BU38" s="7"/>
+      <c r="BV38" s="7"/>
+      <c r="BW38" s="7"/>
+      <c r="BX38" s="7"/>
+      <c r="BY38" s="7"/>
+      <c r="BZ38" s="7"/>
+      <c r="CA38" s="7"/>
+      <c r="CB38" s="7"/>
+      <c r="CC38" s="7"/>
+      <c r="CD38" s="7"/>
+      <c r="CE38" s="7"/>
+      <c r="CF38" s="7"/>
+      <c r="CG38" s="7"/>
+      <c r="CH38" s="7"/>
+      <c r="CI38" s="7"/>
+      <c r="CJ38" s="7"/>
+      <c r="CK38" s="7"/>
+      <c r="CL38" s="7"/>
+      <c r="CM38" s="7"/>
+      <c r="CN38" s="7"/>
+      <c r="CO38" s="7"/>
+      <c r="CP38" s="7"/>
+      <c r="CQ38" s="7"/>
+      <c r="CR38" s="7"/>
+      <c r="CS38" s="7"/>
+      <c r="CT38" s="7"/>
+      <c r="CU38" s="7"/>
+      <c r="CV38" s="7"/>
+      <c r="CW38" s="7"/>
+      <c r="CX38" s="7"/>
+      <c r="CY38" s="7"/>
+      <c r="CZ38" s="7"/>
+      <c r="DA38" s="7"/>
+      <c r="DB38" s="7"/>
+      <c r="DC38" s="7"/>
+      <c r="DD38" s="7"/>
+      <c r="DE38" s="7"/>
+      <c r="DF38" s="7"/>
+      <c r="DG38" s="7"/>
+      <c r="DH38" s="7"/>
+      <c r="DI38" s="7"/>
+      <c r="DJ38" s="7"/>
+      <c r="DK38" s="7"/>
+      <c r="DL38" s="7"/>
+      <c r="DM38" s="7"/>
+      <c r="DN38" s="7"/>
+      <c r="DO38" s="7"/>
+      <c r="DP38" s="7"/>
+      <c r="DQ38" s="7"/>
+      <c r="DR38" s="7"/>
+    </row>
+    <row r="39" customFormat="false" ht="26.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="29"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="5"/>
+    </row>
+    <row r="40" customFormat="false" ht="22.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="30"/>
+      <c r="B40" s="31"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="31"/>
+      <c r="F40" s="31"/>
+      <c r="G40" s="31"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="33"/>
+      <c r="J40" s="33"/>
       <c r="K40" s="5"/>
     </row>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="30"/>
+      <c r="B41" s="31"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
+      <c r="E41" s="31"/>
+      <c r="F41" s="31"/>
+      <c r="G41" s="31"/>
+      <c r="H41" s="31"/>
+      <c r="I41" s="33"/>
+      <c r="J41" s="33"/>
+      <c r="K41" s="5"/>
+    </row>
+    <row r="42" customFormat="false" ht="22.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="34"/>
+      <c r="B42" s="35"/>
+      <c r="C42" s="35"/>
+      <c r="D42" s="35"/>
+      <c r="E42" s="35"/>
+      <c r="F42" s="35"/>
+      <c r="G42" s="35"/>
+      <c r="H42" s="35"/>
+      <c r="I42" s="35"/>
+      <c r="J42" s="35"/>
+      <c r="K42" s="5"/>
+    </row>
+    <row r="43" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="36"/>
+      <c r="B43" s="37"/>
+      <c r="C43" s="37"/>
+      <c r="D43" s="37"/>
+      <c r="E43" s="37"/>
+      <c r="F43" s="37"/>
+      <c r="G43" s="37"/>
+      <c r="H43" s="38"/>
+      <c r="I43" s="38"/>
+      <c r="J43" s="38"/>
+      <c r="K43" s="5"/>
+    </row>
+    <row r="44" customFormat="false" ht="24.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="39"/>
+      <c r="B44" s="40"/>
+      <c r="C44" s="40"/>
+      <c r="D44" s="40"/>
+      <c r="E44" s="40"/>
+      <c r="F44" s="40"/>
+      <c r="G44" s="40"/>
+      <c r="H44" s="40"/>
+      <c r="I44" s="41"/>
+      <c r="J44" s="41"/>
+      <c r="K44" s="5"/>
+    </row>
+    <row r="45" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="34"/>
+      <c r="B45" s="35"/>
+      <c r="C45" s="35"/>
+      <c r="D45" s="35"/>
+      <c r="E45" s="35"/>
+      <c r="F45" s="35"/>
+      <c r="G45" s="35"/>
+      <c r="H45" s="35"/>
+      <c r="I45" s="42"/>
+      <c r="J45" s="35"/>
+      <c r="K45" s="5"/>
+    </row>
+    <row r="46" customFormat="false" ht="16.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="36"/>
+      <c r="B46" s="37"/>
+      <c r="C46" s="37"/>
+      <c r="D46" s="37"/>
+      <c r="E46" s="37"/>
+      <c r="F46" s="37"/>
+      <c r="G46" s="37"/>
+      <c r="H46" s="38"/>
+      <c r="I46" s="38"/>
+      <c r="J46" s="38"/>
+      <c r="K46" s="5"/>
+    </row>
+    <row r="47" customFormat="false" ht="24.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="43"/>
+      <c r="B47" s="35"/>
+      <c r="C47" s="35"/>
+      <c r="D47" s="35"/>
+      <c r="E47" s="35"/>
+      <c r="F47" s="35"/>
+      <c r="G47" s="35"/>
+      <c r="H47" s="35"/>
+      <c r="I47" s="35"/>
+      <c r="J47" s="35"/>
+      <c r="K47" s="5"/>
+    </row>
+    <row r="48" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="36"/>
+      <c r="B48" s="37"/>
+      <c r="C48" s="37"/>
+      <c r="D48" s="37"/>
+      <c r="E48" s="37"/>
+      <c r="F48" s="37"/>
+      <c r="G48" s="37"/>
+      <c r="H48" s="38"/>
+      <c r="I48" s="38"/>
+      <c r="J48" s="38"/>
+      <c r="K48" s="5"/>
+    </row>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5"/>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
+    </row>
     <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
done changes to excel formatting
</commit_message>
<xml_diff>
--- a/reports/sample/sample-monthly-ip-report.xlsx
+++ b/reports/sample/sample-monthly-ip-report.xlsx
@@ -113,10 +113,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
-    <numFmt numFmtId="166" formatCode="&quot;$ &quot;#,##0,&quot; K&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.00%"/>
+    <numFmt numFmtId="167" formatCode="&quot;$ &quot;#,##0,&quot; K&quot;"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -280,7 +281,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -329,6 +330,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -385,15 +390,19 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -401,19 +410,19 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -977,19 +986,19 @@
       <c r="DO3" s="7"/>
       <c r="DP3" s="7"/>
       <c r="DQ3" s="7"/>
-      <c r="DS3" s="0"/>
+      <c r="DS3" s="12"/>
     </row>
     <row r="4" s="11" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="9"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="14"/>
       <c r="K4" s="5"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
@@ -1101,7 +1110,7 @@
       <c r="DO4" s="7"/>
       <c r="DP4" s="7"/>
       <c r="DQ4" s="7"/>
-      <c r="DS4" s="0"/>
+      <c r="DS4" s="12"/>
     </row>
     <row r="5" s="11" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8"/>
@@ -1235,135 +1244,135 @@
       <c r="DO5" s="7"/>
       <c r="DP5" s="7"/>
       <c r="DQ5" s="7"/>
-      <c r="DS5" s="0"/>
+      <c r="DS5" s="12"/>
     </row>
     <row r="6" s="7" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14"/>
-      <c r="B6" s="15" t="n">
+      <c r="A6" s="15"/>
+      <c r="B6" s="16" t="n">
         <v>43</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15" t="n">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="16" t="n">
         <v>33</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="16" t="n">
         <v>92</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="16" t="n">
         <v>35</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16" t="n">
+      <c r="I6" s="17"/>
+      <c r="J6" s="17" t="n">
         <v>224</v>
       </c>
       <c r="K6" s="5"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
-      <c r="DS6" s="0"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+      <c r="DS6" s="12"/>
     </row>
     <row r="7" s="7" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14"/>
-      <c r="B7" s="18" t="n">
+      <c r="A7" s="15"/>
+      <c r="B7" s="19" t="n">
         <v>41</v>
       </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18" t="n">
+      <c r="C7" s="19"/>
+      <c r="D7" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>89</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="19" t="n">
         <v>46</v>
       </c>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18" t="n">
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19" t="n">
         <v>233</v>
       </c>
       <c r="K7" s="5"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
-      <c r="P7" s="17"/>
-      <c r="DS7" s="0"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
+      <c r="DS7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14"/>
-      <c r="B8" s="18" t="n">
+      <c r="A8" s="15"/>
+      <c r="B8" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18" t="n">
+      <c r="C8" s="19"/>
+      <c r="D8" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>41</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>74</v>
       </c>
-      <c r="G8" s="18" t="n">
+      <c r="G8" s="19" t="n">
         <v>56</v>
       </c>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18" t="n">
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19" t="n">
         <v>207</v>
       </c>
       <c r="K8" s="5"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
-      <c r="O8" s="17"/>
-      <c r="P8" s="17"/>
+      <c r="L8" s="18"/>
+      <c r="M8" s="18"/>
+      <c r="N8" s="18"/>
+      <c r="O8" s="18"/>
+      <c r="P8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14"/>
-      <c r="B9" s="18" t="n">
+      <c r="A9" s="15"/>
+      <c r="B9" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>53</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <v>66</v>
       </c>
-      <c r="G9" s="18" t="n">
+      <c r="G9" s="19" t="n">
         <v>57</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18" t="n">
+      <c r="I9" s="19"/>
+      <c r="J9" s="19" t="n">
         <v>218</v>
       </c>
       <c r="K9" s="5"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="17"/>
-      <c r="P9" s="17"/>
+      <c r="L9" s="18"/>
+      <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
@@ -1379,11 +1388,11 @@
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
       <c r="K10" s="5"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="17"/>
-      <c r="O10" s="17"/>
-      <c r="P10" s="17"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
@@ -1414,123 +1423,123 @@
       <c r="K12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14"/>
-      <c r="B13" s="15" t="n">
+      <c r="A13" s="15"/>
+      <c r="B13" s="16" t="n">
         <v>53</v>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="16" t="n">
         <v>55</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="16" t="n">
         <v>147</v>
       </c>
-      <c r="G13" s="15" t="n">
+      <c r="G13" s="16" t="n">
         <v>75</v>
       </c>
-      <c r="H13" s="16" t="n">
+      <c r="H13" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="I13" s="16"/>
-      <c r="J13" s="16" t="n">
+      <c r="I13" s="17"/>
+      <c r="J13" s="17" t="n">
         <v>367</v>
       </c>
       <c r="K13" s="5"/>
     </row>
     <row r="14" s="7" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14"/>
-      <c r="B14" s="19" t="n">
+      <c r="A14" s="15"/>
+      <c r="B14" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="C14" s="19" t="n">
+      <c r="C14" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="E14" s="19" t="n">
+      <c r="E14" s="20" t="n">
         <v>60</v>
       </c>
-      <c r="F14" s="19" t="n">
+      <c r="F14" s="20" t="n">
         <v>142</v>
       </c>
-      <c r="G14" s="19" t="n">
+      <c r="G14" s="20" t="n">
         <v>90</v>
       </c>
-      <c r="H14" s="19" t="n">
+      <c r="H14" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="I14" s="19"/>
-      <c r="J14" s="20" t="n">
+      <c r="I14" s="20"/>
+      <c r="J14" s="21" t="n">
         <v>394</v>
       </c>
       <c r="K14" s="5"/>
-      <c r="DS14" s="0"/>
+      <c r="DS14" s="12"/>
     </row>
     <row r="15" s="7" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14"/>
-      <c r="B15" s="19" t="n">
+      <c r="A15" s="15"/>
+      <c r="B15" s="20" t="n">
         <v>37</v>
       </c>
-      <c r="C15" s="19" t="n">
+      <c r="C15" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="20" t="n">
         <v>40</v>
       </c>
-      <c r="F15" s="19" t="n">
+      <c r="F15" s="20" t="n">
         <v>109</v>
       </c>
-      <c r="G15" s="19" t="n">
+      <c r="G15" s="20" t="n">
         <v>95</v>
       </c>
-      <c r="H15" s="19" t="n">
+      <c r="H15" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="I15" s="19"/>
-      <c r="J15" s="20" t="n">
+      <c r="I15" s="20"/>
+      <c r="J15" s="21" t="n">
         <v>310</v>
       </c>
       <c r="K15" s="5"/>
-      <c r="DS15" s="0"/>
+      <c r="DS15" s="12"/>
     </row>
     <row r="16" s="7" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14"/>
-      <c r="B16" s="21" t="n">
+      <c r="A16" s="15"/>
+      <c r="B16" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="22" t="n">
         <v>9</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="22" t="n">
         <v>9</v>
       </c>
-      <c r="E16" s="21" t="n">
+      <c r="E16" s="22" t="n">
         <v>60</v>
       </c>
-      <c r="F16" s="21" t="n">
+      <c r="F16" s="22" t="n">
         <v>132</v>
       </c>
-      <c r="G16" s="21" t="n">
+      <c r="G16" s="22" t="n">
         <v>123</v>
       </c>
-      <c r="H16" s="21" t="n">
+      <c r="H16" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21" t="n">
+      <c r="I16" s="22"/>
+      <c r="J16" s="22" t="n">
         <v>385</v>
       </c>
       <c r="K16" s="5"/>
-      <c r="DS16" s="0"/>
+      <c r="DS16" s="12"/>
     </row>
     <row r="17" s="7" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
@@ -1562,7 +1571,7 @@
         <v>424</v>
       </c>
       <c r="K17" s="5"/>
-      <c r="DS17" s="0"/>
+      <c r="DS17" s="12"/>
     </row>
     <row r="18" s="7" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6"/>
@@ -1576,32 +1585,32 @@
       <c r="I18" s="6"/>
       <c r="J18" s="6"/>
       <c r="K18" s="5"/>
-      <c r="DS18" s="0"/>
+      <c r="DS18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="21"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="16"/>
+      <c r="A19" s="23"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="25"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="17"/>
       <c r="K19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="16"/>
+      <c r="A20" s="23"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="17"/>
       <c r="K20" s="5"/>
     </row>
     <row r="21" s="7" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1618,69 +1627,69 @@
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
       <c r="K21" s="5"/>
-      <c r="DS21" s="0"/>
+      <c r="DS21" s="12"/>
     </row>
     <row r="22" s="7" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="23"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="20"/>
-      <c r="J22" s="16"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="17"/>
       <c r="K22" s="5"/>
-      <c r="DS22" s="0"/>
+      <c r="DS22" s="12"/>
     </row>
     <row r="23" s="7" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="J23" s="16"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="17"/>
       <c r="K23" s="5"/>
-      <c r="DS23" s="0"/>
+      <c r="DS23" s="12"/>
     </row>
     <row r="24" s="7" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="23"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="20"/>
-      <c r="J24" s="16"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="17"/>
       <c r="K24" s="5"/>
-      <c r="DS24" s="0"/>
+      <c r="DS24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="20"/>
-      <c r="I25" s="20"/>
-      <c r="J25" s="16"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="17"/>
       <c r="K25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1714,48 +1723,48 @@
       <c r="K27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="20"/>
-      <c r="J28" s="16"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="17"/>
       <c r="K28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="18"/>
-      <c r="H29" s="20"/>
-      <c r="I29" s="20"/>
-      <c r="J29" s="16"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="21"/>
+      <c r="J29" s="17"/>
       <c r="K29" s="5"/>
     </row>
     <row r="30" s="11" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="18"/>
-      <c r="H30" s="20"/>
-      <c r="I30" s="20"/>
-      <c r="J30" s="16"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="17"/>
       <c r="K30" s="5"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -1867,21 +1876,21 @@
       <c r="DO30" s="7"/>
       <c r="DP30" s="7"/>
       <c r="DQ30" s="7"/>
-      <c r="DS30" s="0"/>
+      <c r="DS30" s="12"/>
     </row>
     <row r="31" s="11" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="s">
+      <c r="A31" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B31" s="25"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="18"/>
-      <c r="H31" s="20"/>
-      <c r="I31" s="20"/>
-      <c r="J31" s="16"/>
+      <c r="B31" s="26"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="17"/>
       <c r="K31" s="5"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -1993,7 +2002,7 @@
       <c r="DO31" s="7"/>
       <c r="DP31" s="7"/>
       <c r="DQ31" s="7"/>
-      <c r="DS31" s="0"/>
+      <c r="DS31" s="12"/>
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
@@ -2011,16 +2020,16 @@
       <c r="K32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14"/>
-      <c r="B33" s="15"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="15"/>
-      <c r="F33" s="15"/>
-      <c r="G33" s="15"/>
-      <c r="H33" s="15"/>
-      <c r="I33" s="15"/>
-      <c r="J33" s="15"/>
+      <c r="A33" s="15"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="16"/>
+      <c r="I33" s="16"/>
+      <c r="J33" s="16"/>
       <c r="K33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2042,15 +2051,15 @@
       <c r="A35" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="9"/>
+      <c r="B35" s="27"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="27"/>
+      <c r="J35" s="27"/>
       <c r="K35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2178,18 +2187,18 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="8"/>
-      <c r="B37" s="26"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
-      <c r="J37" s="27"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="28"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="29"/>
+      <c r="J37" s="29"/>
       <c r="K37" s="5"/>
-      <c r="L37" s="28"/>
-      <c r="M37" s="28"/>
+      <c r="L37" s="30"/>
+      <c r="M37" s="30"/>
       <c r="N37" s="1"/>
       <c r="O37" s="7"/>
       <c r="P37" s="7"/>
@@ -2426,7 +2435,7 @@
       <c r="DR38" s="7"/>
     </row>
     <row r="39" customFormat="false" ht="26.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="29"/>
+      <c r="A39" s="31"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
@@ -2439,59 +2448,59 @@
       <c r="K39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="22.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="30"/>
-      <c r="B40" s="31"/>
-      <c r="C40" s="31"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="31"/>
-      <c r="F40" s="31"/>
-      <c r="G40" s="31"/>
-      <c r="H40" s="33"/>
-      <c r="I40" s="33"/>
-      <c r="J40" s="33"/>
+      <c r="A40" s="32"/>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="34"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="33"/>
+      <c r="H40" s="35"/>
+      <c r="I40" s="35"/>
+      <c r="J40" s="35"/>
       <c r="K40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="30"/>
-      <c r="B41" s="31"/>
-      <c r="C41" s="31"/>
-      <c r="D41" s="31"/>
-      <c r="E41" s="31"/>
-      <c r="F41" s="31"/>
-      <c r="G41" s="31"/>
-      <c r="H41" s="33"/>
-      <c r="I41" s="33"/>
-      <c r="J41" s="33"/>
+      <c r="A41" s="32"/>
+      <c r="B41" s="33"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="33"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="33"/>
+      <c r="G41" s="33"/>
+      <c r="H41" s="35"/>
+      <c r="I41" s="35"/>
+      <c r="J41" s="35"/>
       <c r="K41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="22.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="8"/>
-      <c r="B42" s="26"/>
-      <c r="C42" s="26"/>
-      <c r="D42" s="26"/>
-      <c r="E42" s="26"/>
-      <c r="F42" s="26"/>
-      <c r="G42" s="26"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="26"/>
-      <c r="J42" s="26"/>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="28"/>
+      <c r="I42" s="28"/>
+      <c r="J42" s="28"/>
       <c r="K42" s="5"/>
     </row>
     <row r="43" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="34"/>
-      <c r="B43" s="35"/>
-      <c r="C43" s="35"/>
-      <c r="D43" s="35"/>
-      <c r="E43" s="35"/>
-      <c r="F43" s="35"/>
-      <c r="G43" s="36"/>
-      <c r="H43" s="36"/>
-      <c r="I43" s="36"/>
-      <c r="J43" s="36"/>
+      <c r="A43" s="36"/>
+      <c r="B43" s="37"/>
+      <c r="C43" s="37"/>
+      <c r="D43" s="37"/>
+      <c r="E43" s="37"/>
+      <c r="F43" s="37"/>
+      <c r="G43" s="38"/>
+      <c r="H43" s="38"/>
+      <c r="I43" s="38"/>
+      <c r="J43" s="38"/>
       <c r="K43" s="5"/>
     </row>
     <row r="44" customFormat="false" ht="24.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="29"/>
+      <c r="A44" s="31"/>
       <c r="B44" s="9"/>
       <c r="C44" s="9"/>
       <c r="D44" s="9"/>
@@ -2505,54 +2514,54 @@
     </row>
     <row r="45" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="8"/>
-      <c r="B45" s="26"/>
-      <c r="C45" s="26"/>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="27"/>
-      <c r="I45" s="27"/>
-      <c r="J45" s="26"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="28"/>
+      <c r="G45" s="28"/>
+      <c r="H45" s="29"/>
+      <c r="I45" s="29"/>
+      <c r="J45" s="28"/>
       <c r="K45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="16.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="34"/>
-      <c r="B46" s="35"/>
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="35"/>
-      <c r="G46" s="36"/>
-      <c r="H46" s="36"/>
-      <c r="I46" s="36"/>
-      <c r="J46" s="36"/>
+      <c r="A46" s="36"/>
+      <c r="B46" s="37"/>
+      <c r="C46" s="37"/>
+      <c r="D46" s="37"/>
+      <c r="E46" s="37"/>
+      <c r="F46" s="37"/>
+      <c r="G46" s="38"/>
+      <c r="H46" s="38"/>
+      <c r="I46" s="38"/>
+      <c r="J46" s="38"/>
       <c r="K46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="24.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="37"/>
-      <c r="B47" s="26"/>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="26"/>
-      <c r="I47" s="26"/>
-      <c r="J47" s="26"/>
+      <c r="A47" s="39"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="28"/>
+      <c r="F47" s="28"/>
+      <c r="G47" s="28"/>
+      <c r="H47" s="28"/>
+      <c r="I47" s="28"/>
+      <c r="J47" s="28"/>
       <c r="K47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="34"/>
-      <c r="B48" s="35"/>
-      <c r="C48" s="35"/>
-      <c r="D48" s="35"/>
-      <c r="E48" s="35"/>
-      <c r="F48" s="35"/>
-      <c r="G48" s="36"/>
-      <c r="H48" s="36"/>
-      <c r="I48" s="36"/>
-      <c r="J48" s="36"/>
+      <c r="A48" s="36"/>
+      <c r="B48" s="37"/>
+      <c r="C48" s="37"/>
+      <c r="D48" s="37"/>
+      <c r="E48" s="37"/>
+      <c r="F48" s="37"/>
+      <c r="G48" s="38"/>
+      <c r="H48" s="38"/>
+      <c r="I48" s="38"/>
+      <c r="J48" s="38"/>
       <c r="K48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
static data feed in progress
</commit_message>
<xml_diff>
--- a/reports/sample/sample-monthly-ip-report.xlsx
+++ b/reports/sample/sample-monthly-ip-report.xlsx
@@ -1114,25 +1114,15 @@
     </row>
     <row r="5" s="11" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8"/>
-      <c r="B5" s="9" t="n">
-        <v>35</v>
-      </c>
+      <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="9" t="n">
-        <v>40</v>
-      </c>
-      <c r="F5" s="9" t="n">
-        <v>85</v>
-      </c>
-      <c r="G5" s="9" t="n">
-        <v>42</v>
-      </c>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
-      <c r="J5" s="10" t="n">
-        <v>202</v>
-      </c>
+      <c r="J5" s="10"/>
       <c r="K5" s="5"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -1248,29 +1238,15 @@
     </row>
     <row r="6" s="7" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15"/>
-      <c r="B6" s="16" t="n">
-        <v>43</v>
-      </c>
+      <c r="B6" s="16"/>
       <c r="C6" s="16"/>
-      <c r="D6" s="16" t="n">
-        <v>13</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <v>33</v>
-      </c>
-      <c r="F6" s="16" t="n">
-        <v>92</v>
-      </c>
-      <c r="G6" s="16" t="n">
-        <v>35</v>
-      </c>
-      <c r="H6" s="17" t="n">
-        <v>3</v>
-      </c>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="17"/>
       <c r="I6" s="17"/>
-      <c r="J6" s="17" t="n">
-        <v>224</v>
-      </c>
+      <c r="J6" s="17"/>
       <c r="K6" s="5"/>
       <c r="L6" s="18"/>
       <c r="M6" s="18"/>
@@ -1281,27 +1257,15 @@
     </row>
     <row r="7" s="7" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15"/>
-      <c r="B7" s="19" t="n">
-        <v>41</v>
-      </c>
+      <c r="B7" s="19"/>
       <c r="C7" s="19"/>
-      <c r="D7" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>39</v>
-      </c>
-      <c r="F7" s="19" t="n">
-        <v>89</v>
-      </c>
-      <c r="G7" s="19" t="n">
-        <v>46</v>
-      </c>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
       <c r="H7" s="19"/>
       <c r="I7" s="19"/>
-      <c r="J7" s="19" t="n">
-        <v>233</v>
-      </c>
+      <c r="J7" s="19"/>
       <c r="K7" s="5"/>
       <c r="L7" s="18"/>
       <c r="M7" s="18"/>
@@ -1312,27 +1276,15 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15"/>
-      <c r="B8" s="19" t="n">
-        <v>25</v>
-      </c>
+      <c r="B8" s="19"/>
       <c r="C8" s="19"/>
-      <c r="D8" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="E8" s="19" t="n">
-        <v>41</v>
-      </c>
-      <c r="F8" s="19" t="n">
-        <v>74</v>
-      </c>
-      <c r="G8" s="19" t="n">
-        <v>56</v>
-      </c>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
       <c r="H8" s="19"/>
       <c r="I8" s="19"/>
-      <c r="J8" s="19" t="n">
-        <v>207</v>
-      </c>
+      <c r="J8" s="19"/>
       <c r="K8" s="5"/>
       <c r="L8" s="18"/>
       <c r="M8" s="18"/>
@@ -1342,31 +1294,15 @@
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15"/>
-      <c r="B9" s="19" t="n">
-        <v>30</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>53</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>66</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>57</v>
-      </c>
-      <c r="H9" s="19" t="n">
-        <v>1</v>
-      </c>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
       <c r="I9" s="19"/>
-      <c r="J9" s="19" t="n">
-        <v>218</v>
-      </c>
+      <c r="J9" s="19"/>
       <c r="K9" s="5"/>
       <c r="L9" s="18"/>
       <c r="M9" s="18"/>
@@ -1424,120 +1360,56 @@
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15"/>
-      <c r="B13" s="16" t="n">
-        <v>53</v>
-      </c>
-      <c r="C13" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="D13" s="16" t="n">
-        <v>19</v>
-      </c>
-      <c r="E13" s="16" t="n">
-        <v>55</v>
-      </c>
-      <c r="F13" s="16" t="n">
-        <v>147</v>
-      </c>
-      <c r="G13" s="16" t="n">
-        <v>75</v>
-      </c>
-      <c r="H13" s="17" t="n">
-        <v>12</v>
-      </c>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="17"/>
       <c r="I13" s="17"/>
-      <c r="J13" s="17" t="n">
-        <v>367</v>
-      </c>
+      <c r="J13" s="17"/>
       <c r="K13" s="5"/>
     </row>
     <row r="14" s="7" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15"/>
-      <c r="B14" s="20" t="n">
-        <v>69</v>
-      </c>
-      <c r="C14" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="D14" s="20" t="n">
-        <v>23</v>
-      </c>
-      <c r="E14" s="20" t="n">
-        <v>60</v>
-      </c>
-      <c r="F14" s="20" t="n">
-        <v>142</v>
-      </c>
-      <c r="G14" s="20" t="n">
-        <v>90</v>
-      </c>
-      <c r="H14" s="20" t="n">
-        <v>6</v>
-      </c>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
       <c r="I14" s="20"/>
-      <c r="J14" s="21" t="n">
-        <v>394</v>
-      </c>
+      <c r="J14" s="21"/>
       <c r="K14" s="5"/>
       <c r="DS14" s="12"/>
     </row>
     <row r="15" s="7" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15"/>
-      <c r="B15" s="20" t="n">
-        <v>37</v>
-      </c>
-      <c r="C15" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="D15" s="20" t="n">
-        <v>23</v>
-      </c>
-      <c r="E15" s="20" t="n">
-        <v>40</v>
-      </c>
-      <c r="F15" s="20" t="n">
-        <v>109</v>
-      </c>
-      <c r="G15" s="20" t="n">
-        <v>95</v>
-      </c>
-      <c r="H15" s="20" t="n">
-        <v>2</v>
-      </c>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
       <c r="I15" s="20"/>
-      <c r="J15" s="21" t="n">
-        <v>310</v>
-      </c>
+      <c r="J15" s="21"/>
       <c r="K15" s="5"/>
       <c r="DS15" s="12"/>
     </row>
     <row r="16" s="7" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15"/>
-      <c r="B16" s="22" t="n">
-        <v>50</v>
-      </c>
-      <c r="C16" s="22" t="n">
-        <v>9</v>
-      </c>
-      <c r="D16" s="22" t="n">
-        <v>9</v>
-      </c>
-      <c r="E16" s="22" t="n">
-        <v>60</v>
-      </c>
-      <c r="F16" s="22" t="n">
-        <v>132</v>
-      </c>
-      <c r="G16" s="22" t="n">
-        <v>123</v>
-      </c>
-      <c r="H16" s="22" t="n">
-        <v>2</v>
-      </c>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
       <c r="I16" s="22"/>
-      <c r="J16" s="22" t="n">
-        <v>385</v>
-      </c>
+      <c r="J16" s="22"/>
       <c r="K16" s="5"/>
       <c r="DS16" s="12"/>
     </row>
@@ -1545,31 +1417,15 @@
       <c r="A17" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="9" t="n">
-        <v>51</v>
-      </c>
-      <c r="C17" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="D17" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <v>57</v>
-      </c>
-      <c r="F17" s="9" t="n">
-        <v>196</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>81</v>
-      </c>
-      <c r="H17" s="10" t="n">
-        <v>11</v>
-      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="10"/>
       <c r="I17" s="10"/>
-      <c r="J17" s="10" t="n">
-        <v>424</v>
-      </c>
+      <c r="J17" s="10"/>
       <c r="K17" s="5"/>
       <c r="DS17" s="12"/>
     </row>

</xml_diff>